<commit_message>
Re-cut Investor & Operations workbooks to $555K/$195K structure
Applied the same 8-cell structural edit the SBA package carries, to both
Azalea_Hospice_Investor_Package.xlsx and Azalea_Hospice_Operations_Dashboard.xlsx:
- Inputs B110=555000, B113=195000
- Inputs A139/B139: opening cash subtracts license (paid at close) -> $372,000
- Debt Schedule A2/A17 titles; C18=0 (license seller note zeroed)
- Cash Flow & BS B34=0 (note liability removed)

Verified by independent recalculation (SBA-only debt service $7,803.05/mo,
license note balance 0, opening cash $372,000) and by diffing the shared engine
tabs against the golden SBA package: 0 differences in both workbooks. Audience
tabs (Returns, Dashboard, etc.) recompute off the engine via live formulas.
Set fullCalcOnLoad on both. Updated model note.

https://claude.ai/code/session_01GAHLyfqLR9bxwN2jm6VjPU
</commit_message>
<xml_diff>
--- a/sba_application/09_financial_model/Azalea_Hospice_Investor_Package.xlsx
+++ b/sba_application/09_financial_model/Azalea_Hospice_Investor_Package.xlsx
@@ -1,24 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Returns" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Investment Options" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Unit Economics" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Sensitivity" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Revenue Model" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Staffing &amp; Payroll" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Operating Budget" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Detailed P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Debt Schedule" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Cash Flow &amp; BS" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Actuals vs Model" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Inputs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment Options" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unit Economics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sensitivity" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Model" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Staffing &amp; Payroll" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Operating Budget" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detailed P&amp;L" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt Schedule" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cash Flow &amp; BS" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Actuals vs Model" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="rhc_tier1">Inputs!$B$5</definedName>
@@ -99,8 +99,8 @@
     <numFmt numFmtId="168" formatCode="0.0000"/>
     <numFmt numFmtId="169" formatCode="#,##0.0;(#,##0.0);&quot;-&quot;"/>
     <numFmt numFmtId="170" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
-    <numFmt numFmtId="171" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="172" formatCode="0.00x;(0.00x);&quot;-&quot;"/>
+    <numFmt numFmtId="171" formatCode="0.00x;(0.00x);&quot;-&quot;"/>
+    <numFmt numFmtId="172" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="173" formatCode="#,##0.00;(#,##0.00);&quot;&quot;"/>
     <numFmt numFmtId="174" formatCode="#,##0.00;(#,##0.00)"/>
   </numFmts>
@@ -231,7 +231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="8">
     <border>
       <left/>
       <right/>
@@ -271,11 +271,44 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="72">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -347,7 +380,7 @@
     <xf numFmtId="167" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -365,7 +398,7 @@
     <xf numFmtId="165" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -418,7 +451,7 @@
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="171" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -450,13 +483,26 @@
     <xf numFmtId="174" fontId="6" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="172" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="171" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -3467,7 +3513,7 @@
         </is>
       </c>
       <c r="B110" s="9" t="n">
-        <v>500000</v>
+        <v>555000</v>
       </c>
     </row>
     <row r="111">
@@ -3497,7 +3543,7 @@
         </is>
       </c>
       <c r="B113" s="9" t="n">
-        <v>250000</v>
+        <v>195000</v>
       </c>
     </row>
     <row r="114">
@@ -3715,11 +3761,11 @@
     <row r="139">
       <c r="A139" s="12" t="inlineStr">
         <is>
-          <t>Opening cash = equity + loan - startup - capex</t>
+          <t>Opening cash = equity + loan - startup - capex - license (paid at close)</t>
         </is>
       </c>
       <c r="B139" s="23">
-        <f>Inputs!$B$113+Inputs!$B$110-Inputs!$B$138-Inputs!$B$117</f>
+        <f>Inputs!$B$113+Inputs!$B$110-Inputs!$B$138-Inputs!$B$117-Inputs!$B$120</f>
         <v/>
       </c>
     </row>
@@ -3738,10 +3784,10 @@
   <mergeCells count="18">
     <mergeCell ref="A2:V2"/>
     <mergeCell ref="A16:V16"/>
+    <mergeCell ref="A35:V35"/>
     <mergeCell ref="A137:V137"/>
+    <mergeCell ref="A90:V90"/>
     <mergeCell ref="A76:V76"/>
-    <mergeCell ref="A90:V90"/>
-    <mergeCell ref="A109:V109"/>
     <mergeCell ref="A85:V85"/>
     <mergeCell ref="A1:V1"/>
     <mergeCell ref="A80:V80"/>
@@ -3751,7 +3797,7 @@
     <mergeCell ref="A27:V27"/>
     <mergeCell ref="A105:V105"/>
     <mergeCell ref="A69:V69"/>
-    <mergeCell ref="A35:V35"/>
+    <mergeCell ref="A109:V109"/>
     <mergeCell ref="A4:V4"/>
     <mergeCell ref="A24:V24"/>
   </mergeCells>
@@ -3804,7 +3850,7 @@
     <row r="2" ht="14" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Debt Schedule - SBA 7(a) + Hickory license seller note | Combined DSCR shown (target &gt;= 1.25x)</t>
+          <t>Debt Schedule - SBA 7(a) only (seller paid at close) | DSCR shown (target &gt;= 1.25x)</t>
         </is>
       </c>
     </row>
@@ -4407,7 +4453,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>HICKORY LICENSE SELLER NOTE ($300K, 6%, 36 mo)</t>
+          <t>HICKORY LICENSE - PAID AT CLOSE (no seller note; schedule zeroed)</t>
         </is>
       </c>
     </row>
@@ -4417,9 +4463,8 @@
           <t>Beginning balance</t>
         </is>
       </c>
-      <c r="C18" s="26">
-        <f>Inputs!$B$120</f>
-        <v/>
+      <c r="C18" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="D18" s="24">
         <f>C22</f>
@@ -5207,83 +5252,83 @@
           <t>COMBINED DSCR (period)</t>
         </is>
       </c>
-      <c r="C29" s="62">
+      <c r="C29" s="71">
         <f>IF(C27=0,0,C28/C27)</f>
         <v/>
       </c>
-      <c r="D29" s="62">
+      <c r="D29" s="71">
         <f>IF(D27=0,0,D28/D27)</f>
         <v/>
       </c>
-      <c r="E29" s="62">
+      <c r="E29" s="71">
         <f>IF(E27=0,0,E28/E27)</f>
         <v/>
       </c>
-      <c r="F29" s="62">
+      <c r="F29" s="71">
         <f>IF(F27=0,0,F28/F27)</f>
         <v/>
       </c>
-      <c r="G29" s="62">
+      <c r="G29" s="71">
         <f>IF(G27=0,0,G28/G27)</f>
         <v/>
       </c>
-      <c r="H29" s="62">
+      <c r="H29" s="71">
         <f>IF(H27=0,0,H28/H27)</f>
         <v/>
       </c>
-      <c r="I29" s="62">
+      <c r="I29" s="71">
         <f>IF(I27=0,0,I28/I27)</f>
         <v/>
       </c>
-      <c r="J29" s="62">
+      <c r="J29" s="71">
         <f>IF(J27=0,0,J28/J27)</f>
         <v/>
       </c>
-      <c r="K29" s="62">
+      <c r="K29" s="71">
         <f>IF(K27=0,0,K28/K27)</f>
         <v/>
       </c>
-      <c r="L29" s="62">
+      <c r="L29" s="71">
         <f>IF(L27=0,0,L28/L27)</f>
         <v/>
       </c>
-      <c r="M29" s="62">
+      <c r="M29" s="71">
         <f>IF(M27=0,0,M28/M27)</f>
         <v/>
       </c>
-      <c r="N29" s="62">
+      <c r="N29" s="71">
         <f>IF(N27=0,0,N28/N27)</f>
         <v/>
       </c>
-      <c r="O29" s="62">
+      <c r="O29" s="71">
         <f>IF(O27=0,0,O28/O27)</f>
         <v/>
       </c>
-      <c r="P29" s="62">
+      <c r="P29" s="71">
         <f>IF(P27=0,0,P28/P27)</f>
         <v/>
       </c>
-      <c r="Q29" s="62">
+      <c r="Q29" s="71">
         <f>IF(Q27=0,0,Q28/Q27)</f>
         <v/>
       </c>
-      <c r="R29" s="62">
+      <c r="R29" s="71">
         <f>IF(R27=0,0,R28/R27)</f>
         <v/>
       </c>
-      <c r="S29" s="62">
+      <c r="S29" s="71">
         <f>IF(S27=0,0,S28/S27)</f>
         <v/>
       </c>
-      <c r="T29" s="62">
+      <c r="T29" s="71">
         <f>IF(T27=0,0,T28/T27)</f>
         <v/>
       </c>
-      <c r="U29" s="62">
+      <c r="U29" s="71">
         <f>IF(U27=0,0,U28/U27)</f>
         <v/>
       </c>
-      <c r="V29" s="62">
+      <c r="V29" s="71">
         <f>IF(V27=0,0,V28/V27)</f>
         <v/>
       </c>
@@ -7646,9 +7691,8 @@
           <t>Hickory license note balance</t>
         </is>
       </c>
-      <c r="B34" s="26">
-        <f>Inputs!$B$120</f>
-        <v/>
+      <c r="B34" s="26" t="n">
+        <v>0</v>
       </c>
       <c r="C34" s="26">
         <f>'Debt Schedule'!C22</f>
@@ -8582,7 +8626,7 @@
           <t>Exit EBITDA multiple</t>
         </is>
       </c>
-      <c r="B5" s="25" t="n">
+      <c r="B5" s="67" t="n">
         <v>5</v>
       </c>
     </row>
@@ -8707,7 +8751,7 @@
           <t>MOIC (gross multiple)</t>
         </is>
       </c>
-      <c r="B16" s="31">
+      <c r="B16" s="68">
         <f>SUM(C12:E12)/$B$6</f>
         <v/>
       </c>
@@ -8813,7 +8857,7 @@
           <t>Exit EBITDA multiple</t>
         </is>
       </c>
-      <c r="B7" s="25" t="n">
+      <c r="B7" s="67" t="n">
         <v>5</v>
       </c>
     </row>
@@ -9171,15 +9215,15 @@
           <t>MOIC (gross multiple)</t>
         </is>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="68">
         <f>SUM(C24:G24)/$B$5</f>
         <v/>
       </c>
-      <c r="D32" s="31">
+      <c r="D32" s="68">
         <f>SUM(C25:G25)/$B$5</f>
         <v/>
       </c>
-      <c r="F32" s="31">
+      <c r="F32" s="68">
         <f>SUM(C26:G26)/$B$5</f>
         <v/>
       </c>
@@ -9240,16 +9284,19 @@
           <t>Lowest risk | fixed yield</t>
         </is>
       </c>
+      <c r="C37" s="69" t="n"/>
       <c r="D37" s="37" t="inlineStr">
         <is>
           <t>Medium risk | upside option</t>
         </is>
       </c>
+      <c r="E37" s="69" t="n"/>
       <c r="F37" s="37" t="inlineStr">
         <is>
           <t>Highest risk | highest upside</t>
         </is>
       </c>
+      <c r="G37" s="69" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="20" t="inlineStr">
@@ -9520,10 +9567,10 @@
     <mergeCell ref="F34:G34"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="D31:E31"/>
     <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D31:E31"/>
     <mergeCell ref="F40:G40"/>
-    <mergeCell ref="A43:G43"/>
     <mergeCell ref="B12:C12"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="F12:G12"/>
@@ -10359,83 +10406,83 @@
           <t>Patient-days</t>
         </is>
       </c>
-      <c r="C12" s="50">
+      <c r="C12" s="70">
         <f>C10*C11</f>
         <v/>
       </c>
-      <c r="D12" s="50">
+      <c r="D12" s="70">
         <f>D10*D11</f>
         <v/>
       </c>
-      <c r="E12" s="50">
+      <c r="E12" s="70">
         <f>E10*E11</f>
         <v/>
       </c>
-      <c r="F12" s="50">
+      <c r="F12" s="70">
         <f>F10*F11</f>
         <v/>
       </c>
-      <c r="G12" s="50">
+      <c r="G12" s="70">
         <f>G10*G11</f>
         <v/>
       </c>
-      <c r="H12" s="50">
+      <c r="H12" s="70">
         <f>H10*H11</f>
         <v/>
       </c>
-      <c r="I12" s="50">
+      <c r="I12" s="70">
         <f>I10*I11</f>
         <v/>
       </c>
-      <c r="J12" s="50">
+      <c r="J12" s="70">
         <f>J10*J11</f>
         <v/>
       </c>
-      <c r="K12" s="50">
+      <c r="K12" s="70">
         <f>K10*K11</f>
         <v/>
       </c>
-      <c r="L12" s="50">
+      <c r="L12" s="70">
         <f>L10*L11</f>
         <v/>
       </c>
-      <c r="M12" s="50">
+      <c r="M12" s="70">
         <f>M10*M11</f>
         <v/>
       </c>
-      <c r="N12" s="50">
+      <c r="N12" s="70">
         <f>N10*N11</f>
         <v/>
       </c>
-      <c r="O12" s="50">
+      <c r="O12" s="70">
         <f>O10*O11</f>
         <v/>
       </c>
-      <c r="P12" s="50">
+      <c r="P12" s="70">
         <f>P10*P11</f>
         <v/>
       </c>
-      <c r="Q12" s="50">
+      <c r="Q12" s="70">
         <f>Q10*Q11</f>
         <v/>
       </c>
-      <c r="R12" s="50">
+      <c r="R12" s="70">
         <f>R10*R11</f>
         <v/>
       </c>
-      <c r="S12" s="50">
+      <c r="S12" s="70">
         <f>S10*S11</f>
         <v/>
       </c>
-      <c r="T12" s="50">
+      <c r="T12" s="70">
         <f>T10*T11</f>
         <v/>
       </c>
-      <c r="U12" s="50">
+      <c r="U12" s="70">
         <f>U10*U11</f>
         <v/>
       </c>
-      <c r="V12" s="50">
+      <c r="V12" s="70">
         <f>V10*V11</f>
         <v/>
       </c>

</xml_diff>